<commit_message>
Build site at 2021-04-30 20:01:11 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="224">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -343,7 +343,7 @@
     <t>Deseja solicitar bolsa?</t>
   </si>
   <si>
-    <t>IES da última titulação</t>
+    <t>Nome do Banco</t>
   </si>
   <si>
     <t>Quais as suas expectativas em relação ao curso?</t>
@@ -355,6 +355,12 @@
     <t>Foto para identificação</t>
   </si>
   <si>
+    <t>Agência</t>
+  </si>
+  <si>
+    <t>Conta corrente</t>
+  </si>
+  <si>
     <t>[Document Studio] File Link</t>
   </si>
   <si>
@@ -596,6 +602,87 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1xC4a_QVsrKXPgT_vUInL3mRGZAraVpLx</t>
+  </si>
+  <si>
+    <t>Pateta</t>
+  </si>
+  <si>
+    <t>Solteiro (a)</t>
+  </si>
+  <si>
+    <t>cachorro</t>
+  </si>
+  <si>
+    <t>jljlçjll</t>
+  </si>
+  <si>
+    <t>sdlsdln</t>
+  </si>
+  <si>
+    <t>Disney</t>
+  </si>
+  <si>
+    <t>aBGRHD WET WE</t>
+  </si>
+  <si>
+    <t>llkç</t>
+  </si>
+  <si>
+    <t>knljblj</t>
+  </si>
+  <si>
+    <t>077969</t>
+  </si>
+  <si>
+    <t>9786yh</t>
+  </si>
+  <si>
+    <t>978h9h</t>
+  </si>
+  <si>
+    <t>g7990</t>
+  </si>
+  <si>
+    <t>908gh79</t>
+  </si>
+  <si>
+    <t>97g9</t>
+  </si>
+  <si>
+    <t>9g80y</t>
+  </si>
+  <si>
+    <t>jlnlj</t>
+  </si>
+  <si>
+    <t>jklnljnb</t>
+  </si>
+  <si>
+    <t>1/1/0110</t>
+  </si>
+  <si>
+    <t>lçjlkn</t>
+  </si>
+  <si>
+    <t>Banco do Brasil</t>
+  </si>
+  <si>
+    <t>Boas</t>
+  </si>
+  <si>
+    <t>Empresa onde trabalho</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=10id-u3LIFfWECIvPAxez2XIGtdvkCasJ</t>
+  </si>
+  <si>
+    <t>3299-4</t>
+  </si>
+  <si>
+    <t>213411-4</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1mf6ttqY0wl4s6SPtMMojRU5rD3aFs5If</t>
   </si>
 </sst>
 </file>
@@ -879,7 +966,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="125" width="21.57"/>
+    <col customWidth="1" min="1" max="127" width="21.57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1228,7 +1315,7 @@
       <c r="DK1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="DL1" s="1" t="s">
+      <c r="DL1" s="2" t="s">
         <v>110</v>
       </c>
       <c r="DM1" s="1" t="s">
@@ -1240,14 +1327,20 @@
       <c r="DO1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="DP1" s="3" t="s">
+      <c r="DP1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="DQ1" s="3" t="s">
+      <c r="DQ1" s="2" t="s">
         <v>115</v>
       </c>
       <c r="DR1" s="3" t="s">
         <v>116</v>
+      </c>
+      <c r="DS1" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="DT1" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2">
@@ -1255,25 +1348,25 @@
         <v>44316.478505127314</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I2" s="3">
         <v>0.0</v>
@@ -1282,10 +1375,10 @@
         <v>28034.0</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M2" s="3">
         <v>3.452356354E9</v>
@@ -1294,49 +1387,49 @@
         <v>5.2342334E7</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Q2" s="3">
         <v>1176388.0</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="U2" s="3">
         <v>2542414.0</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="W2" s="3">
         <v>4.5465765E7</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AC2" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AD2" s="3">
         <v>8.71871871E8</v>
@@ -1345,10 +1438,10 @@
         <v>2.354245234E9</v>
       </c>
       <c r="AF2" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="AG2" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AH2" s="5">
         <v>37622.0</v>
@@ -1357,13 +1450,13 @@
         <v>37987.0</v>
       </c>
       <c r="AJ2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="AK2" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="AM2" s="5">
         <v>37987.0</v>
@@ -1372,80 +1465,82 @@
         <v>38353.0</v>
       </c>
       <c r="AO2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AY2" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="AZ2" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BA2" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BB2" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BC2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="BD2" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="BE2" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BF2" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BG2" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="BH2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="BR2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CP2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="CQ2" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="CR2" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="CS2" s="5">
         <v>41764.0</v>
       </c>
       <c r="CU2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DJ2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DK2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="DL2" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="DM2" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="DN2" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="DO2" s="6"/>
-      <c r="DP2" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="DQ2" s="8" t="str">
+      <c r="DP2" s="6"/>
+      <c r="DQ2" s="6"/>
+      <c r="DR2" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="DS2" s="8" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1u2anZ0EbHjDsofd2dRkM3GfGOdyDncPk","Modelo de inscrição.pdf")</f>
         <v>Modelo de inscrição.pdf</v>
       </c>
-      <c r="DR2" s="8" t="str">
+      <c r="DT2" s="8" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179232f4abeddd7c","Email sent to luizeleno@gmail.com, luizeleno@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, luizeleno@usp.br</v>
       </c>
@@ -1455,25 +1550,25 @@
         <v>44316.5262440625</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I3" s="3">
         <v>0.0</v>
@@ -1482,10 +1577,10 @@
         <v>28034.0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M3" s="3">
         <v>9.76986968E8</v>
@@ -1497,46 +1592,46 @@
         <v>28034.0</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U3" s="3">
         <v>7.8979876E7</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="Z3" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AB3" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="AC3" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="AD3" s="3">
         <v>678969.0</v>
@@ -1545,10 +1640,10 @@
         <v>969769.0</v>
       </c>
       <c r="AF3" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="AG3" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AH3" s="5">
         <v>36892.0</v>
@@ -1557,55 +1652,57 @@
         <v>37257.0</v>
       </c>
       <c r="AJ3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AY3" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="AZ3" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BA3" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="BB3" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BC3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="BR3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CP3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DJ3" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DK3" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="DL3" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="DM3" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="DN3" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="DO3" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="DP3" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="DQ3" s="8" t="str">
+        <v>173</v>
+      </c>
+      <c r="DP3" s="6"/>
+      <c r="DQ3" s="6"/>
+      <c r="DR3" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="DS3" s="8" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=16NGZxkX54BKkFKnOroyP0GZY07N5DwVO","Modelo de inscrição.pdf")</f>
         <v>Modelo de inscrição.pdf</v>
       </c>
-      <c r="DR3" s="8" t="str">
+      <c r="DT3" s="8" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179236e4a909c715","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
@@ -1615,25 +1712,25 @@
         <v>44316.534864409725</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I4" s="3">
         <v>9.0</v>
@@ -1642,10 +1739,10 @@
         <v>36892.0</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="M4" s="3">
         <v>2.452345245234E12</v>
@@ -1654,13 +1751,13 @@
         <v>2.452345245234E12</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="R4" s="3">
         <v>2.452345245234E12</v>
@@ -1669,13 +1766,13 @@
         <v>2.452345245234E12</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U4" s="3">
         <v>2.452345245234E12</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="W4" s="3">
         <v>2.452345245234E12</v>
@@ -1717,55 +1814,57 @@
         <v>40238.0</v>
       </c>
       <c r="AJ4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AY4" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AZ4" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BA4" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BB4" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="BC4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="BR4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CP4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DJ4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DK4" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="DL4" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="DM4" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="DN4" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="DO4" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="DP4" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="DQ4" s="8" t="str">
+        <v>187</v>
+      </c>
+      <c r="DP4" s="6"/>
+      <c r="DQ4" s="6"/>
+      <c r="DR4" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="DS4" s="8" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=19adellV69XeNi0ddV8_wkzBGpyWzIBMB","Modelo de inscrição.pdf")</f>
         <v>Modelo de inscrição.pdf</v>
       </c>
-      <c r="DR4" s="8" t="str">
+      <c r="DT4" s="8" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179237987dc737fb","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
@@ -1775,25 +1874,25 @@
         <v>44316.54722596065</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I5" s="3">
         <v>7.0</v>
@@ -1802,7 +1901,7 @@
         <v>2.0</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="L5" s="3">
         <v>425245.0</v>
@@ -1832,7 +1931,7 @@
         <v>425245.0</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="W5" s="3">
         <v>425245.0</v>
@@ -1868,75 +1967,245 @@
         <v>425245.0</v>
       </c>
       <c r="AH5" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AI5" s="5">
         <v>40179.0</v>
       </c>
       <c r="AJ5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AY5" s="3">
         <v>425245.0</v>
       </c>
       <c r="AZ5" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BA5" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BB5" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="BC5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="BR5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CP5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DJ5" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="DK5" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="DL5" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="DM5" s="3">
         <v>425245.0</v>
       </c>
       <c r="DN5" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="DO5" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="DP5" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="DQ5" s="8" t="str">
+        <v>195</v>
+      </c>
+      <c r="DP5" s="6"/>
+      <c r="DQ5" s="6"/>
+      <c r="DR5" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="DS5" s="8" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1xC4a_QVsrKXPgT_vUInL3mRGZAraVpLx","Modelo de inscrição.pdf")</f>
         <v>Modelo de inscrição.pdf</v>
       </c>
-      <c r="DR5" s="8" t="str">
+      <c r="DT5" s="8" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1792389e62950452","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>44316.6378121875</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J6" s="5">
+        <v>43556.0</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="M6" s="3">
+        <v>346356.0</v>
+      </c>
+      <c r="N6" s="3">
+        <v>23556.0</v>
+      </c>
+      <c r="O6" s="5">
+        <v>44197.0</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>2354453.0</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="U6" s="3">
+        <v>980970.0</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="W6" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="Z6" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="AA6" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="AD6" s="3">
+        <v>76879.0</v>
+      </c>
+      <c r="AE6" s="3">
+        <v>98589.0</v>
+      </c>
+      <c r="AF6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="AG6" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="AH6" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="AI6" s="5">
+        <v>40909.0</v>
+      </c>
+      <c r="AJ6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY6" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="AZ6" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="BA6" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="BB6" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BC6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ6" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="DK6" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="DL6" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="DM6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="DN6" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="DO6" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="DP6" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="DQ6" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="DR6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="DS6" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1mf6ttqY0wl4s6SPtMMojRU5rD3aFs5If","Modelo de inscrição.pdf")</f>
+        <v>Modelo de inscrição.pdf</v>
+      </c>
+      <c r="DT6" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17924016727f959e","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="DP2"/>
+    <hyperlink r:id="rId1" ref="DR2"/>
     <hyperlink r:id="rId2" ref="DO3"/>
-    <hyperlink r:id="rId3" ref="DP3"/>
+    <hyperlink r:id="rId3" ref="DR3"/>
     <hyperlink r:id="rId4" ref="DO4"/>
-    <hyperlink r:id="rId5" ref="DP4"/>
+    <hyperlink r:id="rId5" ref="DR4"/>
     <hyperlink r:id="rId6" ref="DO5"/>
-    <hyperlink r:id="rId7" ref="DP5"/>
+    <hyperlink r:id="rId7" ref="DR5"/>
+    <hyperlink r:id="rId8" ref="DO6"/>
+    <hyperlink r:id="rId9" ref="DR6"/>
   </hyperlinks>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-05 14:01:39 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="258">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -683,6 +683,108 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1mf6ttqY0wl4s6SPtMMojRU5rD3aFs5If</t>
+  </si>
+  <si>
+    <t>Fábio Cavassani Notz</t>
+  </si>
+  <si>
+    <t>fcnotz@gmail.com</t>
+  </si>
+  <si>
+    <t>Resende</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro/Brasil</t>
+  </si>
+  <si>
+    <t>05711873741</t>
+  </si>
+  <si>
+    <t>Detran</t>
+  </si>
+  <si>
+    <t>Rua Manoel da Silva Torres - 555</t>
+  </si>
+  <si>
+    <t>Alegria</t>
+  </si>
+  <si>
+    <t>Mariana</t>
+  </si>
+  <si>
+    <t>Esposa</t>
+  </si>
+  <si>
+    <t>AEDB - CPGE - Centro de Pesquisa Pos Graduação e Extensão</t>
+  </si>
+  <si>
+    <t>Engenharia da Qualidade/Pos Graduação</t>
+  </si>
+  <si>
+    <t>AEDB - Faculdade de Engenharia de Resende</t>
+  </si>
+  <si>
+    <t>Engenharia de Produção Automotiva/Graduação</t>
+  </si>
+  <si>
+    <t>Colégio Municipal Getúlio Vargas</t>
+  </si>
+  <si>
+    <t>Técnico Mecânica Industrial/Ensino Técnico</t>
+  </si>
+  <si>
+    <t>Volkswagen Caminhões e Ônibus</t>
+  </si>
+  <si>
+    <t>Engenheiro do Produto Pleno</t>
+  </si>
+  <si>
+    <t>Privada</t>
+  </si>
+  <si>
+    <t>IVM Semcon Automotive</t>
+  </si>
+  <si>
+    <t>Cooper Standard Automotive</t>
+  </si>
+  <si>
+    <t>Assistente Técnico de Qualidade</t>
+  </si>
+  <si>
+    <t>Aumentar meu conhecimento em materiais e poder disseminar as técnicas utilizadas na academia dentro da área profissinal, aumentando o nível de conhecimento técnico dos profissionais de engenharia. Dessa forma, podemos utilizar o que há de mais recente em pesquisas para projetar itens robustos e reduzir insumos que impactam o meio ambiente e a sociedade em um todo.</t>
+  </si>
+  <si>
+    <t>Outros</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1m37ygvAQWzQC3hLjM7bW6Rgw1DFK8j5t</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1yWUHn-YIQ_2Bee5YONBKvGLLHaRiWugr</t>
+  </si>
+  <si>
+    <t>RJ/Brasil</t>
+  </si>
+  <si>
+    <t>Marian</t>
+  </si>
+  <si>
+    <t>Pós Graduação / Engenharia da Qualidade</t>
+  </si>
+  <si>
+    <t>Graduação / Engenharia de Prdoução Automotiva</t>
+  </si>
+  <si>
+    <t>Ensino Médio Técnico /Mecânica Industrial</t>
+  </si>
+  <si>
+    <t>Aumentar meu conhecimento em materiais e poder disseminar as técnicas utilizadas na academia dentro da área profissional, aumentando o nível de conhecimento técnico dos profissionais de engenharia. Dessa forma, podemos utilizar o que há de mais recente em pesquisas para projetar itens robustos e reduzir insumos que impactam o meio ambiente e a sociedade em um todo.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=19Zr1JtA_wYet4QT8uwMBNggAOhe4iqhN</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1gYvSEDZHnK391EA_7oG1THNiqctrWftt</t>
   </si>
 </sst>
 </file>
@@ -2194,6 +2296,482 @@
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>44321.36374539352</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J7" s="5">
+        <v>31117.0</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="N7" s="3">
+        <v>1.30556871E8</v>
+      </c>
+      <c r="O7" s="5">
+        <v>37602.0</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>1.1389273E7</v>
+      </c>
+      <c r="R7" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="U7" s="3">
+        <v>2.7524108E7</v>
+      </c>
+      <c r="V7" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="W7" s="3">
+        <v>2.4999241932E10</v>
+      </c>
+      <c r="X7" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="Y7" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="Z7" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="AA7" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="AC7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="AD7" s="3">
+        <v>2.7524108E7</v>
+      </c>
+      <c r="AE7" s="3">
+        <v>2.4999782216E10</v>
+      </c>
+      <c r="AF7" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="AG7" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="AH7" s="5">
+        <v>43285.0</v>
+      </c>
+      <c r="AI7" s="5">
+        <v>43871.0</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK7" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="AL7" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="AM7" s="5">
+        <v>38750.0</v>
+      </c>
+      <c r="AN7" s="5">
+        <v>40522.0</v>
+      </c>
+      <c r="AO7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AP7" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="AQ7" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="AR7" s="5">
+        <v>36558.0</v>
+      </c>
+      <c r="AS7" s="5">
+        <v>37965.0</v>
+      </c>
+      <c r="AT7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY7" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="AZ7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BA7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BB7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BC7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BS7" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="BT7" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="BU7" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="BV7" s="5">
+        <v>43325.0</v>
+      </c>
+      <c r="BX7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BY7" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="BZ7" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="CA7" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="CB7" s="5">
+        <v>40834.0</v>
+      </c>
+      <c r="CC7" s="5">
+        <v>43322.0</v>
+      </c>
+      <c r="CD7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="CE7" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="CF7" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="CG7" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="CH7" s="5">
+        <v>39483.0</v>
+      </c>
+      <c r="CI7" s="5">
+        <v>40831.0</v>
+      </c>
+      <c r="CJ7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DM7" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="DN7" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="DO7" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="DR7" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="DS7" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1yWUHn-YIQ_2Bee5YONBKvGLLHaRiWugr","Fábio Cavassani Notz-MESTRADO.pdf")</f>
+        <v>Fábio Cavassani Notz-MESTRADO.pdf</v>
+      </c>
+      <c r="DT7" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1793c57d5b5d33e9","Email sent to fcnotz@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to fcnotz@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>44321.37839172454</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J8" s="5">
+        <v>31117.0</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="N8" s="3">
+        <v>1.30556871E8</v>
+      </c>
+      <c r="O8" s="5">
+        <v>37617.0</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>1.1389273E7</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="U8" s="3">
+        <v>2.7524108E7</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="W8" s="3">
+        <v>2.4999241932E10</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="Z8" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="AA8" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="AC8" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="AD8" s="3">
+        <v>2.7524108E7</v>
+      </c>
+      <c r="AE8" s="3">
+        <v>2.4999782216E10</v>
+      </c>
+      <c r="AF8" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="AG8" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="AH8" s="5">
+        <v>43285.0</v>
+      </c>
+      <c r="AI8" s="5">
+        <v>43871.0</v>
+      </c>
+      <c r="AJ8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK8" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="AL8" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM8" s="5">
+        <v>38750.0</v>
+      </c>
+      <c r="AN8" s="5">
+        <v>40522.0</v>
+      </c>
+      <c r="AO8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="AQ8" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="AR8" s="5">
+        <v>36558.0</v>
+      </c>
+      <c r="AS8" s="5">
+        <v>37965.0</v>
+      </c>
+      <c r="AT8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY8" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="AZ8" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BA8" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BB8" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="BC8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BS8" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="BT8" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="BU8" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="BV8" s="5">
+        <v>43325.0</v>
+      </c>
+      <c r="BX8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BY8" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="BZ8" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="CA8" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="CB8" s="5">
+        <v>40834.0</v>
+      </c>
+      <c r="CC8" s="5">
+        <v>43322.0</v>
+      </c>
+      <c r="CD8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="CE8" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="CF8" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="CG8" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="CH8" s="5">
+        <v>39483.0</v>
+      </c>
+      <c r="CI8" s="5">
+        <v>40831.0</v>
+      </c>
+      <c r="CJ8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DM8" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="DN8" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="DO8" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="DR8" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="DS8" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1gYvSEDZHnK391EA_7oG1THNiqctrWftt","Fábio Cavassani Notz-MESTRADO.pdf")</f>
+        <v>Fábio Cavassani Notz-MESTRADO.pdf</v>
+      </c>
+      <c r="DT8" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1793c6b1d517576a","Email sent to fcnotz@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to fcnotz@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DR2"/>
@@ -2205,7 +2783,11 @@
     <hyperlink r:id="rId7" ref="DR5"/>
     <hyperlink r:id="rId8" ref="DO6"/>
     <hyperlink r:id="rId9" ref="DR6"/>
+    <hyperlink r:id="rId10" ref="DO7"/>
+    <hyperlink r:id="rId11" ref="DR7"/>
+    <hyperlink r:id="rId12" ref="DO8"/>
+    <hyperlink r:id="rId13" ref="DR8"/>
   </hyperlinks>
-  <drawing r:id="rId10"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-20 22:01:32 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="199">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -497,6 +497,120 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1gYvSEDZHnK391EA_7oG1THNiqctrWftt</t>
+  </si>
+  <si>
+    <t>Adolfo Luiz de Souza</t>
+  </si>
+  <si>
+    <t>adolfo_luiz@hotmail.com</t>
+  </si>
+  <si>
+    <t>Solteiro (a)</t>
+  </si>
+  <si>
+    <t>Parda</t>
+  </si>
+  <si>
+    <t>Volta Redonda</t>
+  </si>
+  <si>
+    <t>Rua Luis Romanelli N°80 Apart 201</t>
+  </si>
+  <si>
+    <t>Regina Célia</t>
+  </si>
+  <si>
+    <t>Cruzeiro</t>
+  </si>
+  <si>
+    <t>Lucinéia Rosa de Souza</t>
+  </si>
+  <si>
+    <t>Mãe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua Emilio de Menezes N°28 </t>
+  </si>
+  <si>
+    <t>Eucaliptal</t>
+  </si>
+  <si>
+    <t>Universidade Federal Fluminense</t>
+  </si>
+  <si>
+    <t>Bacharel em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>Senai - Rj</t>
+  </si>
+  <si>
+    <t>Técnico em Eletromecânica</t>
+  </si>
+  <si>
+    <t>Colégio Plural de Ensino médio</t>
+  </si>
+  <si>
+    <t>Técnico deInformática</t>
+  </si>
+  <si>
+    <t>Espanhol</t>
+  </si>
+  <si>
+    <t>Intermediário</t>
+  </si>
+  <si>
+    <t>Básico</t>
+  </si>
+  <si>
+    <t>Greenbrier Maxion</t>
+  </si>
+  <si>
+    <t>Analista de Laboratório</t>
+  </si>
+  <si>
+    <t>UCD (Universidade daIrlanda)</t>
+  </si>
+  <si>
+    <t>Técnico de Laboratório</t>
+  </si>
+  <si>
+    <t>Iochpe Maxion</t>
+  </si>
+  <si>
+    <t>Estagiário em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>CSN</t>
+  </si>
+  <si>
+    <t>Lider de produção</t>
+  </si>
+  <si>
+    <t>Vest Pré - Vestibular</t>
+  </si>
+  <si>
+    <t>Professor ( fisica e matemática)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitor - Algebra </t>
+  </si>
+  <si>
+    <t>Autonomo</t>
+  </si>
+  <si>
+    <t>Professor de Inglês</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Buscar ainda mais conhecimento na área de materiais;
+*interatividade com os colegas;
+*troca de experiências na prática de atuação;
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1PTziYvry07P5qBBHLWfRMd3nn-gyRUDF</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1neJchzbxRh3bfdX3KsBaVavFrfQW70fB</t>
   </si>
 </sst>
 </file>
@@ -1630,13 +1744,322 @@
         <v>Email sent to fcnotz@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>44336.72752872686</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J4" s="5">
+        <v>31551.0</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="M4" s="3">
+        <v>1.2139481771E10</v>
+      </c>
+      <c r="N4" s="3">
+        <v>2.09298199E8</v>
+      </c>
+      <c r="O4" s="5">
+        <v>39511.0</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="U4" s="3">
+        <v>1.270541E7</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W4" s="3">
+        <v>2.4998136459E10</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="AA4" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="AC4" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AD4" s="3">
+        <v>2.726402E7</v>
+      </c>
+      <c r="AE4" s="3">
+        <v>2.4981684477E10</v>
+      </c>
+      <c r="AF4" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="AG4" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="AH4" s="5">
+        <v>40605.0</v>
+      </c>
+      <c r="AI4" s="5">
+        <v>42802.0</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AK4" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="AL4" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AM4" s="5">
+        <v>39115.0</v>
+      </c>
+      <c r="AN4" s="5">
+        <v>39784.0</v>
+      </c>
+      <c r="AO4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AP4" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="AQ4" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AR4" s="5">
+        <v>38022.0</v>
+      </c>
+      <c r="AS4" s="5">
+        <v>39061.0</v>
+      </c>
+      <c r="AT4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AZ4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BA4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BB4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD4" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="BE4" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF4" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="BG4" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BH4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BS4" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="BT4" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="BU4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BV4" s="5">
+        <v>44221.0</v>
+      </c>
+      <c r="BX4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BZ4" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="CA4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CB4" s="5">
+        <v>43525.0</v>
+      </c>
+      <c r="CC4" s="5">
+        <v>43768.0</v>
+      </c>
+      <c r="CD4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CE4" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="CF4" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="CG4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH4" s="5">
+        <v>42217.0</v>
+      </c>
+      <c r="CI4" s="5">
+        <v>42765.0</v>
+      </c>
+      <c r="CJ4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CK4" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="CL4" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="CM4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CN4" s="5">
+        <v>43221.0</v>
+      </c>
+      <c r="CO4" s="5">
+        <v>43311.0</v>
+      </c>
+      <c r="CP4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CQ4" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="CR4" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="CS4" s="5">
+        <v>41308.0</v>
+      </c>
+      <c r="CT4" s="5">
+        <v>41718.0</v>
+      </c>
+      <c r="CU4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CV4" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="CW4" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="CX4" s="5">
+        <v>40577.0</v>
+      </c>
+      <c r="CY4" s="5">
+        <v>40942.0</v>
+      </c>
+      <c r="CZ4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="DA4" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="DB4" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="DC4" s="5">
+        <v>43831.0</v>
+      </c>
+      <c r="DE4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DM4" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="DN4" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="DO4" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="DR4" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="DS4" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1neJchzbxRh3bfdX3KsBaVavFrfQW70fB","Adolfo Luiz de Souza-MESTRADO.pdf")</f>
+        <v>Adolfo Luiz de Souza-MESTRADO.pdf</v>
+      </c>
+      <c r="DT4" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798b76df5665db5","Email sent to adolfo_luiz@hotmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to adolfo_luiz@hotmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
     <hyperlink r:id="rId2" ref="DR2"/>
     <hyperlink r:id="rId3" ref="DO3"/>
     <hyperlink r:id="rId4" ref="DR3"/>
+    <hyperlink r:id="rId5" ref="DO4"/>
+    <hyperlink r:id="rId6" ref="DR4"/>
   </hyperlinks>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-31 19:01:04 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="218">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -611,6 +611,63 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1neJchzbxRh3bfdX3KsBaVavFrfQW70fB</t>
+  </si>
+  <si>
+    <t>Karoline Elerbrock Borowski</t>
+  </si>
+  <si>
+    <t>karoline.borowski@usp.br</t>
+  </si>
+  <si>
+    <t>Feminino</t>
+  </si>
+  <si>
+    <t>Lorena</t>
+  </si>
+  <si>
+    <t>SP - Brasil</t>
+  </si>
+  <si>
+    <t>SSP</t>
+  </si>
+  <si>
+    <t>Avenida Capitão Messias Ribeiro, N°384</t>
+  </si>
+  <si>
+    <t>Olaria</t>
+  </si>
+  <si>
+    <t>Julienne Maria Fiorentini Elerbrock</t>
+  </si>
+  <si>
+    <t>Universidade de São Paulo, Escola de Engenharia de Lorena</t>
+  </si>
+  <si>
+    <t>Engenheira de Materiais</t>
+  </si>
+  <si>
+    <t>Francês</t>
+  </si>
+  <si>
+    <t>Banco do Brasil</t>
+  </si>
+  <si>
+    <t>Espero aprofundar meus conhecimentos adquiridos na graduação e me tornar mais independente para conduzir uma pesquisa, em um curso de excelência.</t>
+  </si>
+  <si>
+    <t>Escola onde estudo</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1IhqQqIIXLBro1NPZ99apEAtcRqg8tcXq</t>
+  </si>
+  <si>
+    <t>857-5</t>
+  </si>
+  <si>
+    <t>118968-9</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1r_QdjaGdSJ42jx1jFW7KWlPb_7LHfIvP</t>
   </si>
 </sst>
 </file>
@@ -2051,6 +2108,187 @@
         <v>Email sent to adolfo_luiz@hotmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>44347.61737568287</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J5" s="5">
+        <v>35605.0</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="M5" s="3">
+        <v>3.7759045816E10</v>
+      </c>
+      <c r="N5" s="3">
+        <v>4.70557783E8</v>
+      </c>
+      <c r="O5" s="5">
+        <v>42432.0</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>9269646.0</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="U5" s="3">
+        <v>1.260702E7</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W5" s="3">
+        <v>1.299737357E10</v>
+      </c>
+      <c r="X5" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="Y5" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z5" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="AC5" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="AD5" s="3">
+        <v>1.260702E7</v>
+      </c>
+      <c r="AE5" s="3">
+        <v>1.2997897578E10</v>
+      </c>
+      <c r="AF5" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="AG5" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="AH5" s="5">
+        <v>42039.0</v>
+      </c>
+      <c r="AI5" s="5">
+        <v>44406.0</v>
+      </c>
+      <c r="AJ5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY5" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AZ5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BA5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BB5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD5" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="BE5" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF5" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BG5" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BH5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="DL5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="DM5" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="DN5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="DO5" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="DP5" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="DQ5" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="DR5" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="DS5" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1r_QdjaGdSJ42jx1jFW7KWlPb_7LHfIvP","Karoline Elerbrock Borowski-MESTRADO.pdf")</f>
+        <v>Karoline Elerbrock Borowski-MESTRADO.pdf</v>
+      </c>
+      <c r="DT5" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179c38b8c8c5f888","Email sent to karoline.borowski@usp.br, ppgem-eel@usp.br")</f>
+        <v>Email sent to karoline.borowski@usp.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -2059,7 +2297,9 @@
     <hyperlink r:id="rId4" ref="DR3"/>
     <hyperlink r:id="rId5" ref="DO4"/>
     <hyperlink r:id="rId6" ref="DR4"/>
+    <hyperlink r:id="rId7" ref="DO5"/>
+    <hyperlink r:id="rId8" ref="DR5"/>
   </hyperlinks>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-06-04 12:30:35 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="241">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -668,6 +668,75 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1r_QdjaGdSJ42jx1jFW7KWlPb_7LHfIvP</t>
+  </si>
+  <si>
+    <t>BRUNO NERY STOCO</t>
+  </si>
+  <si>
+    <t>nerystoco@gmail.com</t>
+  </si>
+  <si>
+    <t>VOLTA REDONDA</t>
+  </si>
+  <si>
+    <t>RIO DE JANEIRO/BRASIL</t>
+  </si>
+  <si>
+    <t>DETRAN</t>
+  </si>
+  <si>
+    <t>RUA G 147</t>
+  </si>
+  <si>
+    <t>VALE DO SOL</t>
+  </si>
+  <si>
+    <t>PINHEIRAL</t>
+  </si>
+  <si>
+    <t>CINTIA</t>
+  </si>
+  <si>
+    <t>ESPOSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSIDADE FEDERAL FLUMINENSE </t>
+  </si>
+  <si>
+    <t>ENGENHEIRO METALURGISTA</t>
+  </si>
+  <si>
+    <t>INGLES</t>
+  </si>
+  <si>
+    <t>TERNIUM BRASIL</t>
+  </si>
+  <si>
+    <t>CONSULTOR</t>
+  </si>
+  <si>
+    <t>RHIMAGNESITA</t>
+  </si>
+  <si>
+    <t>ASSISTENTE TÉCNICO</t>
+  </si>
+  <si>
+    <t>ASSOCIAÇÃO BRASILEIRA DE SOLDAGEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROFESSOR TEMPORÁRIO </t>
+  </si>
+  <si>
+    <t>AUMENTAR MEU CONHECIMENTO TÉCNICO EM REFRATÁRIO PARA APLICAÇÃO NA INDUSTRIA</t>
+  </si>
+  <si>
+    <t>Empresa onde trabalho</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1qX1f7jE6JvxCws2JSEwuerWsajepI4Pq</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1_UDdAxob4UOwtCZktaHw1dUvzoJ2PPNQ</t>
   </si>
 </sst>
 </file>
@@ -2289,6 +2358,208 @@
         <v>Email sent to karoline.borowski@usp.br, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>44350.82845410879</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I6" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="J6" s="5">
+        <v>31427.0</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="M6" s="3">
+        <v>1.1070069701E10</v>
+      </c>
+      <c r="N6" s="3">
+        <v>1.16832569E8</v>
+      </c>
+      <c r="O6" s="5">
+        <v>41769.0</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="U6" s="3">
+        <v>2.7197E7</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W6" s="3">
+        <v>2.1967520232E10</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="Z6" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA6" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="AD6" s="3">
+        <v>2.7197E7</v>
+      </c>
+      <c r="AE6" s="3">
+        <v>2.498859485E10</v>
+      </c>
+      <c r="AF6" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="AG6" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="AH6" s="5">
+        <v>38534.0</v>
+      </c>
+      <c r="AI6" s="5">
+        <v>40162.0</v>
+      </c>
+      <c r="AJ6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY6" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="AZ6" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BA6" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BB6" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR6" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BS6" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT6" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="BU6" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BV6" s="5">
+        <v>42659.0</v>
+      </c>
+      <c r="BX6" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY6" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="BZ6" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="CA6" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CB6" s="5">
+        <v>40103.0</v>
+      </c>
+      <c r="CC6" s="5">
+        <v>42655.0</v>
+      </c>
+      <c r="CD6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP6" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CQ6" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="CR6" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="CS6" s="5">
+        <v>39934.0</v>
+      </c>
+      <c r="CT6" s="5">
+        <v>40167.0</v>
+      </c>
+      <c r="CU6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DM6" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="DN6" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="DO6" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="DR6" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="DS6" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1_UDdAxob4UOwtCZktaHw1dUvzoJ2PPNQ","BRUNO NERY STOCO-MESTRADO.pdf")</f>
+        <v>BRUNO NERY STOCO-MESTRADO.pdf</v>
+      </c>
+      <c r="DT6" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179d414d7854f0b9","Email sent to nerystoco@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to nerystoco@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -2299,7 +2570,9 @@
     <hyperlink r:id="rId6" ref="DR4"/>
     <hyperlink r:id="rId7" ref="DO5"/>
     <hyperlink r:id="rId8" ref="DR5"/>
+    <hyperlink r:id="rId9" ref="DO6"/>
+    <hyperlink r:id="rId10" ref="DR6"/>
   </hyperlinks>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-06-07 12:31:46 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="263">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -737,6 +737,72 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1_UDdAxob4UOwtCZktaHw1dUvzoJ2PPNQ</t>
+  </si>
+  <si>
+    <t>Luiz Felipe Ribeiro Rabelo</t>
+  </si>
+  <si>
+    <t>luiz.feliperibeiroo@gmail.com</t>
+  </si>
+  <si>
+    <t>Não declarado</t>
+  </si>
+  <si>
+    <t>Magé</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Rua Tupi</t>
+  </si>
+  <si>
+    <t>Vila Hepacare</t>
+  </si>
+  <si>
+    <t>Fernando Luiz Rabelo</t>
+  </si>
+  <si>
+    <t>Pai</t>
+  </si>
+  <si>
+    <t>Av. Simão da Mota</t>
+  </si>
+  <si>
+    <t>Centro</t>
+  </si>
+  <si>
+    <t>Faculdade de Tecnologia de Pindamonhangaba</t>
+  </si>
+  <si>
+    <t>Tecnólogo - Processos de soldagem</t>
+  </si>
+  <si>
+    <t>AECI mining explosives</t>
+  </si>
+  <si>
+    <t>Estágiario</t>
+  </si>
+  <si>
+    <t>Nubank</t>
+  </si>
+  <si>
+    <t>Contribuir para o desenvolvimento da educação e pesquisa nacional no Programa de Pós Graduação em Engenharia de Materiais.</t>
+  </si>
+  <si>
+    <t>Pesquisa online</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1V7WB_7pg-Eg0dVsrxZCPx9F52Mfh3dZ-</t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>1399738-0</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1RF0mw-MY-pObM2F263N849fk3r72QopV</t>
   </si>
 </sst>
 </file>
@@ -2560,6 +2626,187 @@
         <v>Email sent to nerystoco@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>44353.8931380787</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J7" s="5">
+        <v>35653.0</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="M7" s="3">
+        <v>1.2856892752E10</v>
+      </c>
+      <c r="N7" s="3">
+        <v>2.8981945E8</v>
+      </c>
+      <c r="O7" s="5">
+        <v>42356.0</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="R7" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="U7" s="3">
+        <v>1.2608345E7</v>
+      </c>
+      <c r="V7" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W7" s="3">
+        <v>2.1980350805E10</v>
+      </c>
+      <c r="X7" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="Y7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="Z7" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="AA7" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="AB7" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="AC7" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="AD7" s="3">
+        <v>2.5900001E7</v>
+      </c>
+      <c r="AE7" s="3">
+        <v>2.1967746172E10</v>
+      </c>
+      <c r="AF7" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="AG7" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH7" s="5">
+        <v>43313.0</v>
+      </c>
+      <c r="AI7" s="5">
+        <v>44166.0</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY7" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AZ7" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BA7" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BB7" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BC7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR7" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BS7" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="BT7" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="BU7" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BV7" s="5">
+        <v>44319.0</v>
+      </c>
+      <c r="BW7" s="5">
+        <v>44350.0</v>
+      </c>
+      <c r="BX7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK7" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="DL7" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="DM7" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="DN7" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="DO7" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="DP7" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="DQ7" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="DR7" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="DS7" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1RF0mw-MY-pObM2F263N849fk3r72QopV","Luiz Felipe Ribeiro Rabelo-MESTRADO.pdf")</f>
+        <v>Luiz Felipe Ribeiro Rabelo-MESTRADO.pdf</v>
+      </c>
+      <c r="DT7" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179e3dd4b59324f8","Email sent to luiz.feliperibeiroo@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to luiz.feliperibeiroo@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -2572,7 +2819,9 @@
     <hyperlink r:id="rId8" ref="DR5"/>
     <hyperlink r:id="rId9" ref="DO6"/>
     <hyperlink r:id="rId10" ref="DR6"/>
+    <hyperlink r:id="rId11" ref="DO7"/>
+    <hyperlink r:id="rId12" ref="DR7"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-06-09 15:31:14 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="290">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -803,6 +803,87 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1RF0mw-MY-pObM2F263N849fk3r72QopV</t>
+  </si>
+  <si>
+    <t>Daniel Lucas Feliciano</t>
+  </si>
+  <si>
+    <t>nielluc@yahoo.com.br</t>
+  </si>
+  <si>
+    <t>MONTES CLAROS</t>
+  </si>
+  <si>
+    <t>MG/BRASIL</t>
+  </si>
+  <si>
+    <t>06686263648</t>
+  </si>
+  <si>
+    <t>SSPMG</t>
+  </si>
+  <si>
+    <t>RUA VISCONDE DE PINDAMONHANGABA, 111</t>
+  </si>
+  <si>
+    <t>JARDIM BOA VISTA</t>
+  </si>
+  <si>
+    <t>PINDAMONHANGABA</t>
+  </si>
+  <si>
+    <t>DANIELA MASSULA</t>
+  </si>
+  <si>
+    <t>SP/BRASIL</t>
+  </si>
+  <si>
+    <t>UNIVERSIDADE FEDERAL DE ITAJUBÁ</t>
+  </si>
+  <si>
+    <t>ENGENHARIA HÍDRICA</t>
+  </si>
+  <si>
+    <t>FUNDAÇÃO GETULIO VARGAS</t>
+  </si>
+  <si>
+    <t>MBA EM GESTÃO DE PROJETOS</t>
+  </si>
+  <si>
+    <t>INGLÊS</t>
+  </si>
+  <si>
+    <t>ESPANHOL</t>
+  </si>
+  <si>
+    <t>Novelis do Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Engenheiro de Desenvolvimento de Produto</t>
+  </si>
+  <si>
+    <t>Engenheiro de Assistência Técnica</t>
+  </si>
+  <si>
+    <t>Tenaris Confab</t>
+  </si>
+  <si>
+    <t>Engenheiro de Serviços de Campo</t>
+  </si>
+  <si>
+    <t>Analista de Gestão Industrial</t>
+  </si>
+  <si>
+    <t>Aprofundar meus conhecimentos na área de engenharia de materiais e aplicá-los na minha área profissional, e futuramente, na área acadêmica.</t>
+  </si>
+  <si>
+    <t>Aluno PPGEM</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1OT47jj3ANgHuv8EU3xviCVa-mIqVZKBu</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1brYFB2tkdfor9cAB3IJpFYIQ-wvhrRKc</t>
   </si>
 </sst>
 </file>
@@ -2807,6 +2888,259 @@
         <v>Email sent to luiz.feliperibeiroo@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>44356.42816293982</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I8" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="J8" s="5">
+        <v>30607.0</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="N8" s="3">
+        <v>1.2487025E7</v>
+      </c>
+      <c r="O8" s="5">
+        <v>39049.0</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>1.1390615E7</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="U8" s="3">
+        <v>1.2401011E7</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W8" s="3">
+        <v>1.2988179612E10</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="Z8" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA8" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="AC8" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="AD8" s="3">
+        <v>1.2401011E7</v>
+      </c>
+      <c r="AE8" s="3">
+        <v>1.2981317772E10</v>
+      </c>
+      <c r="AF8" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="AG8" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="AH8" s="5">
+        <v>37681.0</v>
+      </c>
+      <c r="AI8" s="5">
+        <v>39814.0</v>
+      </c>
+      <c r="AJ8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AK8" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="AL8" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="AM8" s="5">
+        <v>40664.0</v>
+      </c>
+      <c r="AN8" s="5">
+        <v>41394.0</v>
+      </c>
+      <c r="AO8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY8" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="AZ8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BA8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BB8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD8" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="BE8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BF8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BG8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BH8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BS8" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="BT8" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="BU8" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BV8" s="5">
+        <v>43435.0</v>
+      </c>
+      <c r="BX8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY8" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="BZ8" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="CA8" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CB8" s="5">
+        <v>42352.0</v>
+      </c>
+      <c r="CC8" s="5">
+        <v>43435.0</v>
+      </c>
+      <c r="CD8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CE8" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="CF8" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="CG8" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH8" s="5">
+        <v>41518.0</v>
+      </c>
+      <c r="CI8" s="5">
+        <v>42308.0</v>
+      </c>
+      <c r="CJ8" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CK8" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="CL8" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="CM8" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CN8" s="5">
+        <v>40848.0</v>
+      </c>
+      <c r="CO8" s="5">
+        <v>41455.0</v>
+      </c>
+      <c r="CP8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DM8" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="DN8" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="DO8" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="DR8" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="DS8" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1brYFB2tkdfor9cAB3IJpFYIQ-wvhrRKc","Daniel Lucas Feliciano-MESTRADO.pdf")</f>
+        <v>Daniel Lucas Feliciano-MESTRADO.pdf</v>
+      </c>
+      <c r="DT8" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/179f0eb3e5070647","Email sent to nielluc@yahoo.com.br, ppgem-eel@usp.br")</f>
+        <v>Email sent to nielluc@yahoo.com.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -2821,7 +3155,9 @@
     <hyperlink r:id="rId10" ref="DR6"/>
     <hyperlink r:id="rId11" ref="DO7"/>
     <hyperlink r:id="rId12" ref="DR7"/>
+    <hyperlink r:id="rId13" ref="DO8"/>
+    <hyperlink r:id="rId14" ref="DR8"/>
   </hyperlinks>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-06-21 22:00:37 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
+++ b/_Drive/Formularios/Mestrado-DoutoradoDireto/Inscrição para Mestrado e Doutorado Direto (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="319">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -884,6 +884,93 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1brYFB2tkdfor9cAB3IJpFYIQ-wvhrRKc</t>
+  </si>
+  <si>
+    <t>Guilherme Eduardo Silva Magalhães</t>
+  </si>
+  <si>
+    <t>engmagalhaes.guilherme@gmail.com</t>
+  </si>
+  <si>
+    <t>Osasco</t>
+  </si>
+  <si>
+    <t>Brasil</t>
+  </si>
+  <si>
+    <t>SSP/SP</t>
+  </si>
+  <si>
+    <t>Av. Hilário Pereira de Souza, 492</t>
+  </si>
+  <si>
+    <t>06010170</t>
+  </si>
+  <si>
+    <t>Carlos Magalhães</t>
+  </si>
+  <si>
+    <t>Estrada da Grama, 500</t>
+  </si>
+  <si>
+    <t>Saboó</t>
+  </si>
+  <si>
+    <t>São Roque</t>
+  </si>
+  <si>
+    <t>São Paulo</t>
+  </si>
+  <si>
+    <t>Universidade Santa Cecília - UNISANTA</t>
+  </si>
+  <si>
+    <t>Bacharelado em Engenharia Mecânica</t>
+  </si>
+  <si>
+    <t>Instituto Tecnológico de Barueri - ITB</t>
+  </si>
+  <si>
+    <t>Técnico em Tecnologia da Informação</t>
+  </si>
+  <si>
+    <t>Techno Smart - Comércio e Manutenção de Máquinas</t>
+  </si>
+  <si>
+    <t>Engenheiro de manutenção e projetos</t>
+  </si>
+  <si>
+    <t>Exército Brasileiro - 2º Grupo de Artilharia Antiaérea</t>
+  </si>
+  <si>
+    <t>1º Tenente - Oficial de Comunicações</t>
+  </si>
+  <si>
+    <t>Pública</t>
+  </si>
+  <si>
+    <t>IBM do Brasil</t>
+  </si>
+  <si>
+    <t>Analista de suporte Técnico - Bilingue</t>
+  </si>
+  <si>
+    <t>Itau</t>
+  </si>
+  <si>
+    <t>Obter ferramentas para conseguir alcançar excelência no meio acadêmico e científico, aplicando tais conhecimentos em meu meio profissional, aumentando meus alicerces  técnico e pensamento crítico, impulsionando meu crescimento pessoal e profissional.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=11aMynd_QbktFUAWcTnsxf9YjKv_ADvkX</t>
+  </si>
+  <si>
+    <t>0462</t>
+  </si>
+  <si>
+    <t>079922</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1czIuuP5sUkVvkD2eSI0PZ8KaEvFcG-JV</t>
   </si>
 </sst>
 </file>
@@ -3141,6 +3228,268 @@
         <v>Email sent to nielluc@yahoo.com.br, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>44368.69018887731</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="5">
+        <v>34130.0</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="M9" s="3">
+        <v>3.89812228E10</v>
+      </c>
+      <c r="N9" s="3">
+        <v>3.4760294E8</v>
+      </c>
+      <c r="O9" s="5">
+        <v>43311.0</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>1.2880307E7</v>
+      </c>
+      <c r="R9" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="U9" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="V9" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="W9" s="3">
+        <v>1.195734681E9</v>
+      </c>
+      <c r="X9" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="Y9" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="Z9" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="AA9" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="AB9" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="AC9" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="AD9" s="3">
+        <v>1.8135695E7</v>
+      </c>
+      <c r="AE9" s="3">
+        <v>1.14176115E8</v>
+      </c>
+      <c r="AF9" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="AG9" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="AH9" s="5">
+        <v>41426.0</v>
+      </c>
+      <c r="AI9" s="5">
+        <v>43983.0</v>
+      </c>
+      <c r="AJ9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AK9" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="AL9" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="AM9" s="5">
+        <v>39448.0</v>
+      </c>
+      <c r="AN9" s="5">
+        <v>40513.0</v>
+      </c>
+      <c r="AO9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY9" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AZ9" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BA9" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BB9" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD9" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="BE9" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF9" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BG9" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BH9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BI9" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="BJ9" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="BK9" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="BL9" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="BM9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BS9" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="BT9" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="BU9" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BV9" s="5">
+        <v>44013.0</v>
+      </c>
+      <c r="BX9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY9" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="BZ9" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="CA9" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="CB9" s="5">
+        <v>40940.0</v>
+      </c>
+      <c r="CC9" s="5">
+        <v>44005.0</v>
+      </c>
+      <c r="CD9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="CE9" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="CF9" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="CG9" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH9" s="5">
+        <v>40269.0</v>
+      </c>
+      <c r="CI9" s="5">
+        <v>40483.0</v>
+      </c>
+      <c r="CJ9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="CP9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DJ9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DK9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="DL9" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="DM9" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="DN9" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="DO9" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="DP9" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="DQ9" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="DR9" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="DS9" s="8" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1czIuuP5sUkVvkD2eSI0PZ8KaEvFcG-JV","Guilherme Eduardo Silva Magalhães-MESTRADO.pdf")</f>
+        <v>Guilherme Eduardo Silva Magalhães-MESTRADO.pdf</v>
+      </c>
+      <c r="DT9" s="8" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17a301119939dedc","Email sent to engmagalhaes.guilherme@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to engmagalhaes.guilherme@gmail.com, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -3157,7 +3506,9 @@
     <hyperlink r:id="rId12" ref="DR7"/>
     <hyperlink r:id="rId13" ref="DO8"/>
     <hyperlink r:id="rId14" ref="DR8"/>
+    <hyperlink r:id="rId15" ref="DO9"/>
+    <hyperlink r:id="rId16" ref="DR9"/>
   </hyperlinks>
-  <drawing r:id="rId15"/>
+  <drawing r:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>